<commit_message>
Refine Day 1 explanations and workbook input checks before publication [skip social]
</commit_message>
<xml_diff>
--- a/public/downloads/budget-vs-actual-template.xlsx
+++ b/public/downloads/budget-vs-actual-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank report" sheetId="1" r:id="Rbc81ebdf51e442a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filled example" sheetId="2" r:id="Rcb525c7a226f45fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank report" sheetId="1" r:id="Rd0f1a1a62e964132"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filled example" sheetId="2" r:id="Rf423e9fd80114b09"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -442,11 +442,11 @@
         <x:v>Net revenue</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(INDEX($H$22:$H$33,$B$5)=2,INDEX($B$22:$B$33,$B$5),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(INDEX($H$22:$H$33,$B$5)=2,INDEX($B$22:$B$33,$B$5),"Unreported"),"Invalid period")</x:f>
         <x:v>Unreported</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(INDEX($I$22:$I$33,$B$5)=2,INDEX($D$22:$D$33,$B$5),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(INDEX($I$22:$I$33,$B$5)=2,INDEX($D$22:$D$33,$B$5),"Unreported"),"Invalid period")</x:f>
         <x:v>Unreported</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
@@ -471,11 +471,11 @@
         <x:v>Included expenses</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(INDEX($H$22:$H$33,$B$5)=2,INDEX($C$22:$C$33,$B$5),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(INDEX($H$22:$H$33,$B$5)=2,INDEX($C$22:$C$33,$B$5),"Unreported"),"Invalid period")</x:f>
         <x:v>Unreported</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(INDEX($I$22:$I$33,$B$5)=2,INDEX($E$22:$E$33,$B$5),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(INDEX($I$22:$I$33,$B$5)=2,INDEX($E$22:$E$33,$B$5),"Unreported"),"Invalid period")</x:f>
         <x:v>Unreported</x:v>
       </x:c>
       <x:c r="D10" s="11" t="str">
@@ -579,11 +579,11 @@
         <x:v>Net revenue</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$H$22:$H$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$B$22:$B$33),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$H$22:$H$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$B$22:$B$33),"Unreported"),"Invalid period")</x:f>
         <x:v>Unreported</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$I$22:$I$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$D$22:$D$33),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$I$22:$I$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$D$22:$D$33),"Unreported"),"Invalid period")</x:f>
         <x:v>Unreported</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
@@ -608,11 +608,11 @@
         <x:v>Included expenses</x:v>
       </x:c>
       <x:c r="B16" s="11" t="str">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$H$22:$H$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$C$22:$C$33),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$H$22:$H$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$C$22:$C$33),"Unreported"),"Invalid period")</x:f>
         <x:v>Unreported</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$I$22:$I$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$E$22:$E$33),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$I$22:$I$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$E$22:$E$33),"Unreported"),"Invalid period")</x:f>
         <x:v>Unreported</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
@@ -731,7 +731,7 @@
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="9" t="n">
-        <x:f>DATE($E$5,1,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,1,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46023</x:v>
       </x:c>
       <x:c r="B22" s="10"/>
@@ -758,7 +758,7 @@
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="9" t="n">
-        <x:f>DATE($E$5,2,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,2,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46054</x:v>
       </x:c>
       <x:c r="B23" s="10"/>
@@ -785,7 +785,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="9" t="n">
-        <x:f>DATE($E$5,3,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,3,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46082</x:v>
       </x:c>
       <x:c r="B24" s="10"/>
@@ -812,7 +812,7 @@
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="9" t="n">
-        <x:f>DATE($E$5,4,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,4,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46113</x:v>
       </x:c>
       <x:c r="B25" s="10"/>
@@ -839,7 +839,7 @@
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="9" t="n">
-        <x:f>DATE($E$5,5,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,5,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46143</x:v>
       </x:c>
       <x:c r="B26" s="10"/>
@@ -866,7 +866,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="9" t="n">
-        <x:f>DATE($E$5,6,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,6,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46174</x:v>
       </x:c>
       <x:c r="B27" s="10"/>
@@ -893,7 +893,7 @@
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="9" t="n">
-        <x:f>DATE($E$5,7,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,7,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46204</x:v>
       </x:c>
       <x:c r="B28" s="10"/>
@@ -920,7 +920,7 @@
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="9" t="n">
-        <x:f>DATE($E$5,8,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,8,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46235</x:v>
       </x:c>
       <x:c r="B29" s="10"/>
@@ -947,7 +947,7 @@
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="9" t="n">
-        <x:f>DATE($E$5,9,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,9,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46266</x:v>
       </x:c>
       <x:c r="B30" s="10"/>
@@ -974,7 +974,7 @@
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="9" t="n">
-        <x:f>DATE($E$5,10,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,10,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46296</x:v>
       </x:c>
       <x:c r="B31" s="10"/>
@@ -1001,7 +1001,7 @@
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="9" t="n">
-        <x:f>DATE($E$5,11,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,11,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46327</x:v>
       </x:c>
       <x:c r="B32" s="10"/>
@@ -1028,7 +1028,7 @@
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="9" t="n">
-        <x:f>DATE($E$5,12,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,12,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46357</x:v>
       </x:c>
       <x:c r="B33" s="10"/>
@@ -1360,11 +1360,11 @@
         <x:v>Net revenue</x:v>
       </x:c>
       <x:c r="B9" s="11" t="n">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(INDEX($H$22:$H$33,$B$5)=2,INDEX($B$22:$B$33,$B$5),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(INDEX($H$22:$H$33,$B$5)=2,INDEX($B$22:$B$33,$B$5),"Unreported"),"Invalid period")</x:f>
         <x:v>30000</x:v>
       </x:c>
       <x:c r="C9" s="11" t="n">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(INDEX($I$22:$I$33,$B$5)=2,INDEX($D$22:$D$33,$B$5),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(INDEX($I$22:$I$33,$B$5)=2,INDEX($D$22:$D$33,$B$5),"Unreported"),"Invalid period")</x:f>
         <x:v>28000</x:v>
       </x:c>
       <x:c r="D9" s="11" t="n">
@@ -1389,11 +1389,11 @@
         <x:v>Included expenses</x:v>
       </x:c>
       <x:c r="B10" s="11" t="n">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(INDEX($H$22:$H$33,$B$5)=2,INDEX($C$22:$C$33,$B$5),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(INDEX($H$22:$H$33,$B$5)=2,INDEX($C$22:$C$33,$B$5),"Unreported"),"Invalid period")</x:f>
         <x:v>20000</x:v>
       </x:c>
       <x:c r="C10" s="11" t="n">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(INDEX($I$22:$I$33,$B$5)=2,INDEX($E$22:$E$33,$B$5),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(INDEX($I$22:$I$33,$B$5)=2,INDEX($E$22:$E$33,$B$5),"Unreported"),"Invalid period")</x:f>
         <x:v>21000</x:v>
       </x:c>
       <x:c r="D10" s="11" t="n">
@@ -1497,11 +1497,11 @@
         <x:v>Net revenue</x:v>
       </x:c>
       <x:c r="B15" s="11" t="n">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$H$22:$H$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$B$22:$B$33),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$H$22:$H$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$B$22:$B$33),"Unreported"),"Invalid period")</x:f>
         <x:v>30000</x:v>
       </x:c>
       <x:c r="C15" s="11" t="n">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$I$22:$I$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$D$22:$D$33),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$I$22:$I$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$D$22:$D$33),"Unreported"),"Invalid period")</x:f>
         <x:v>28000</x:v>
       </x:c>
       <x:c r="D15" s="11" t="n">
@@ -1526,11 +1526,11 @@
         <x:v>Included expenses</x:v>
       </x:c>
       <x:c r="B16" s="11" t="n">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$H$22:$H$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$C$22:$C$33),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$H$22:$H$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$C$22:$C$33),"Unreported"),"Invalid period")</x:f>
         <x:v>20000</x:v>
       </x:c>
       <x:c r="C16" s="11" t="n">
-        <x:f>IF(AND(ISNUMBER($B$5),$B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$I$22:$I$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$E$22:$E$33),"Unreported"),"Invalid month")</x:f>
+        <x:f>IF(AND(IF(ISNUMBER($B$5),AND($B$5=INT($B$5),$B$5&gt;=1,$B$5&lt;=12),FALSE),IF(ISNUMBER($E$5),AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),FALSE)),IF(SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$I$22:$I$33)=2*$B$5,SUMIF($A$22:$A$33,"&lt;="&amp;DATE($E$5,$B$5,1),$E$22:$E$33),"Unreported"),"Invalid period")</x:f>
         <x:v>21000</x:v>
       </x:c>
       <x:c r="D16" s="11" t="n">
@@ -1649,7 +1649,7 @@
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="9" t="n">
-        <x:f>DATE($E$5,1,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,1,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46023</x:v>
       </x:c>
       <x:c r="B22" s="10" t="n">
@@ -1684,7 +1684,7 @@
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="9" t="n">
-        <x:f>DATE($E$5,2,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,2,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46054</x:v>
       </x:c>
       <x:c r="B23" s="10" t="n">
@@ -1719,7 +1719,7 @@
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="9" t="n">
-        <x:f>DATE($E$5,3,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,3,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46082</x:v>
       </x:c>
       <x:c r="B24" s="10" t="n">
@@ -1754,7 +1754,7 @@
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="9" t="n">
-        <x:f>DATE($E$5,4,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,4,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46113</x:v>
       </x:c>
       <x:c r="B25" s="10" t="n">
@@ -1785,7 +1785,7 @@
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="9" t="n">
-        <x:f>DATE($E$5,5,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,5,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46143</x:v>
       </x:c>
       <x:c r="B26" s="10" t="n">
@@ -1816,7 +1816,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="9" t="n">
-        <x:f>DATE($E$5,6,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,6,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46174</x:v>
       </x:c>
       <x:c r="B27" s="10" t="n">
@@ -1847,7 +1847,7 @@
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="9" t="n">
-        <x:f>DATE($E$5,7,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,7,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46204</x:v>
       </x:c>
       <x:c r="B28" s="10" t="n">
@@ -1878,7 +1878,7 @@
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="9" t="n">
-        <x:f>DATE($E$5,8,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,8,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46235</x:v>
       </x:c>
       <x:c r="B29" s="10" t="n">
@@ -1909,7 +1909,7 @@
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="9" t="n">
-        <x:f>DATE($E$5,9,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,9,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46266</x:v>
       </x:c>
       <x:c r="B30" s="10" t="n">
@@ -1940,7 +1940,7 @@
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="9" t="n">
-        <x:f>DATE($E$5,10,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,10,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46296</x:v>
       </x:c>
       <x:c r="B31" s="10" t="n">
@@ -1971,7 +1971,7 @@
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="9" t="n">
-        <x:f>DATE($E$5,11,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,11,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46327</x:v>
       </x:c>
       <x:c r="B32" s="10" t="n">
@@ -2002,7 +2002,7 @@
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="9" t="n">
-        <x:f>DATE($E$5,12,1)</x:f>
+        <x:f>IF(ISNUMBER($E$5),IF(AND($E$5=INT($E$5),$E$5&gt;=1900,$E$5&lt;=9999),DATE($E$5,12,1),"Invalid year"),"Invalid year")</x:f>
         <x:v>46357</x:v>
       </x:c>
       <x:c r="B33" s="10" t="n">

</xml_diff>